<commit_message>
add rows in excel
</commit_message>
<xml_diff>
--- a/test-data/WriteInExcel.xlsx
+++ b/test-data/WriteInExcel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t>TCID</t>
   </si>
@@ -31,19 +31,37 @@
     <t>Smoke</t>
   </si>
   <si>
+    <t>Admin88</t>
+  </si>
+  <si>
+    <t>admin123</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>Sanity</t>
+  </si>
+  <si>
+    <t>Admin11</t>
+  </si>
+  <si>
+    <t>admin1</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>UsNam</t>
+  </si>
+  <si>
+    <t>PWD</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
     <t>Admin</t>
-  </si>
-  <si>
-    <t>admin123</t>
-  </si>
-  <si>
-    <t>TC_002</t>
-  </si>
-  <si>
-    <t>Sanity</t>
-  </si>
-  <si>
-    <t>Admin11</t>
   </si>
 </sst>
 </file>
@@ -420,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="15" customWidth="1"/>
@@ -466,6 +484,34 @@
         <v>10</v>
       </c>
       <c r="D3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added final test file
</commit_message>
<xml_diff>
--- a/test-data/WriteInExcel.xlsx
+++ b/test-data/WriteInExcel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
   <si>
     <t>TCID</t>
   </si>
@@ -62,6 +62,18 @@
   </si>
   <si>
     <t>Admin</t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>Admin77</t>
+  </si>
+  <si>
+    <t>TC_006</t>
+  </si>
+  <si>
+    <t>User2</t>
   </si>
 </sst>
 </file>
@@ -438,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="15" customWidth="1"/>
@@ -515,6 +527,34 @@
         <v>7</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>